<commit_message>
Add SOH report for 2026-10-28
</commit_message>
<xml_diff>
--- a/reports/SOH_28_10_2026.xlsx
+++ b/reports/SOH_28_10_2026.xlsx
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>9967</v>
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>11997</v>
@@ -1478,7 +1478,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>10795</v>
+        <v>10759</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>10251</v>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>546</v>
+        <v>530</v>
       </c>
       <c r="E42" s="3" t="n">
         <v>4836</v>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>4156</v>
+        <v>4150</v>
       </c>
       <c r="E55" s="3" t="n">
         <v>12094</v>
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>300</v>
+        <v>276</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>9595</v>
@@ -2290,7 +2290,7 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="E66" s="3" t="n">
         <v>8060</v>
@@ -2318,7 +2318,7 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>1247</v>
+        <v>1243</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>8181</v>
@@ -2374,7 +2374,7 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>10487</v>
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="E71" s="3" t="n">
         <v>3954</v>
@@ -2514,7 +2514,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>8988</v>
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>2351</v>
+        <v>2345</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>8767</v>
@@ -2598,7 +2598,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>18195</v>
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>2504</v>
+        <v>2498</v>
       </c>
       <c r="E90" s="3" t="n">
         <v>7347</v>
@@ -3074,7 +3074,7 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E94" s="3" t="n">
         <v>36976</v>
@@ -3186,7 +3186,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E98" s="3" t="n">
         <v>41871</v>
@@ -3214,7 +3214,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>704</v>
+        <v>695</v>
       </c>
       <c r="E99" s="3" t="n">
         <v>25495</v>
@@ -3858,7 +3858,7 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E122" s="3" t="n">
         <v>9787</v>
@@ -4306,7 +4306,7 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E138" s="3" t="n">
         <v>5570</v>
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E140" s="3" t="n">
         <v>9853</v>
@@ -4782,7 +4782,7 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="E155" s="3" t="n">
         <v>6251</v>
@@ -4838,7 +4838,7 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E157" s="3" t="n">
         <v>8598</v>
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E158" s="3" t="n">
         <v>12992</v>
@@ -5006,7 +5006,7 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>147</v>
+        <v>123</v>
       </c>
       <c r="E163" s="3" t="n">
         <v>8711</v>
@@ -5034,7 +5034,7 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E164" s="3" t="n">
         <v>6376</v>
@@ -5258,7 +5258,7 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>362</v>
+        <v>314</v>
       </c>
       <c r="E172" s="3" t="n">
         <v>6848</v>
@@ -5370,7 +5370,7 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>696</v>
+        <v>660</v>
       </c>
       <c r="E176" s="3" t="n">
         <v>7016</v>
@@ -5426,7 +5426,7 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>329</v>
+        <v>293</v>
       </c>
       <c r="E178" s="3" t="n">
         <v>6934</v>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E191" s="3" t="n">
         <v>20702</v>
@@ -5986,7 +5986,7 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="E198" s="3" t="n">
         <v>12005</v>
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E200" s="3" t="n">
         <v>13995</v>
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="E211" s="3" t="n">
         <v>5157</v>
@@ -6966,7 +6966,7 @@
         </is>
       </c>
       <c r="D233" s="2" t="n">
-        <v>1894</v>
+        <v>1888</v>
       </c>
       <c r="E233" s="3" t="n">
         <v>8446</v>
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E240" s="3" t="n">
         <v>12504</v>
@@ -8538,7 +8538,7 @@
         </is>
       </c>
       <c r="D292" s="2" t="n">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="E292" s="3" t="n">
         <v>1</v>
@@ -8566,7 +8566,7 @@
         </is>
       </c>
       <c r="D293" s="2" t="n">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="E293" s="3" t="n">
         <v>0</v>
@@ -9746,7 +9746,7 @@
         </is>
       </c>
       <c r="D336" s="2" t="n">
-        <v>240</v>
+        <v>216</v>
       </c>
       <c r="E336" s="3" t="n">
         <v>6659</v>
@@ -9802,7 +9802,7 @@
         </is>
       </c>
       <c r="D338" s="2" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="E338" s="3" t="n">
         <v>9239</v>
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="D340" s="2" t="n">
-        <v>864</v>
+        <v>828</v>
       </c>
       <c r="E340" s="3" t="n">
         <v>6593</v>
@@ -9914,7 +9914,7 @@
         </is>
       </c>
       <c r="D342" s="2" t="n">
-        <v>1056</v>
+        <v>1020</v>
       </c>
       <c r="E342" s="3" t="n">
         <v>6718</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="D355" s="2" t="n">
-        <v>769</v>
+        <v>751</v>
       </c>
       <c r="E355" s="3" t="n">
         <v>3000</v>
@@ -10306,7 +10306,7 @@
         </is>
       </c>
       <c r="D356" s="2" t="n">
-        <v>558</v>
+        <v>540</v>
       </c>
       <c r="E356" s="3" t="n">
         <v>3000</v>
@@ -10362,7 +10362,7 @@
         </is>
       </c>
       <c r="D358" s="2" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="E358" s="3" t="n">
         <v>8597</v>
@@ -10474,7 +10474,7 @@
         </is>
       </c>
       <c r="D362" s="2" t="n">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="E362" s="3" t="n">
         <v>4708</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="D363" s="2" t="n">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="E363" s="3" t="n">
         <v>4708</v>
@@ -10530,7 +10530,7 @@
         </is>
       </c>
       <c r="D364" s="2" t="n">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="E364" s="3" t="n">
         <v>4708</v>
@@ -10558,7 +10558,7 @@
         </is>
       </c>
       <c r="D365" s="2" t="n">
-        <v>720</v>
+        <v>635</v>
       </c>
       <c r="E365" s="3" t="n">
         <v>12500</v>
@@ -10586,7 +10586,7 @@
         </is>
       </c>
       <c r="D366" s="2" t="n">
-        <v>361</v>
+        <v>343</v>
       </c>
       <c r="E366" s="3" t="n">
         <v>8000</v>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="D373" s="2" t="n">
-        <v>1313</v>
+        <v>1113</v>
       </c>
       <c r="E373" s="3" t="n">
         <v>40000</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="D375" s="2" t="n">
-        <v>843</v>
+        <v>801</v>
       </c>
       <c r="E375" s="3" t="n">
         <v>40000</v>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D377" s="2" t="n">
-        <v>768</v>
+        <v>726</v>
       </c>
       <c r="E377" s="3" t="n">
         <v>40000</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="D379" s="2" t="n">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="E379" s="3" t="n">
         <v>40000</v>
@@ -11006,7 +11006,7 @@
         </is>
       </c>
       <c r="D381" s="2" t="n">
-        <v>1378</v>
+        <v>1356</v>
       </c>
       <c r="E381" s="3" t="n">
         <v>17000</v>
@@ -11034,7 +11034,7 @@
         </is>
       </c>
       <c r="D382" s="2" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="E382" s="3" t="n">
         <v>48000</v>
@@ -11286,7 +11286,7 @@
         </is>
       </c>
       <c r="D391" s="2" t="n">
-        <v>647</v>
+        <v>637</v>
       </c>
       <c r="E391" s="3" t="n">
         <v>51000</v>
@@ -11314,7 +11314,7 @@
         </is>
       </c>
       <c r="D392" s="2" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E392" s="3" t="n">
         <v>26500</v>
@@ -11342,7 +11342,7 @@
         </is>
       </c>
       <c r="D393" s="2" t="n">
-        <v>988</v>
+        <v>962</v>
       </c>
       <c r="E393" s="3" t="n">
         <v>51000</v>
@@ -11398,7 +11398,7 @@
         </is>
       </c>
       <c r="D395" s="2" t="n">
-        <v>1320</v>
+        <v>1310</v>
       </c>
       <c r="E395" s="3" t="n">
         <v>51000</v>
@@ -11426,7 +11426,7 @@
         </is>
       </c>
       <c r="D396" s="2" t="n">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="E396" s="3" t="n">
         <v>26500</v>
@@ -11454,7 +11454,7 @@
         </is>
       </c>
       <c r="D397" s="2" t="n">
-        <v>246</v>
+        <v>217</v>
       </c>
       <c r="E397" s="3" t="n">
         <v>51000</v>
@@ -11482,7 +11482,7 @@
         </is>
       </c>
       <c r="D398" s="2" t="n">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="E398" s="3" t="n">
         <v>26500</v>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="D399" s="2" t="n">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E399" s="3" t="n">
         <v>51000</v>
@@ -11706,7 +11706,7 @@
         </is>
       </c>
       <c r="D406" s="2" t="n">
-        <v>2445</v>
+        <v>2439</v>
       </c>
       <c r="E406" s="3" t="n">
         <v>3500</v>
@@ -11930,7 +11930,7 @@
         </is>
       </c>
       <c r="D414" s="2" t="n">
-        <v>2561</v>
+        <v>2485</v>
       </c>
       <c r="E414" s="3" t="n">
         <v>3876</v>
@@ -11958,7 +11958,7 @@
         </is>
       </c>
       <c r="D415" s="2" t="n">
-        <v>458</v>
+        <v>446</v>
       </c>
       <c r="E415" s="3" t="n">
         <v>7612</v>
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="D416" s="2" t="n">
-        <v>249</v>
+        <v>191</v>
       </c>
       <c r="E416" s="3" t="n">
         <v>9000</v>
@@ -12014,7 +12014,7 @@
         </is>
       </c>
       <c r="D417" s="2" t="n">
-        <v>336</v>
+        <v>288</v>
       </c>
       <c r="E417" s="3" t="n">
         <v>8000</v>
@@ -12042,7 +12042,7 @@
         </is>
       </c>
       <c r="D418" s="2" t="n">
-        <v>1613</v>
+        <v>1499</v>
       </c>
       <c r="E418" s="3" t="n">
         <v>8000</v>
@@ -12098,7 +12098,7 @@
         </is>
       </c>
       <c r="D420" s="2" t="n">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="E420" s="3" t="n">
         <v>8000</v>
@@ -12126,7 +12126,7 @@
         </is>
       </c>
       <c r="D421" s="2" t="n">
-        <v>291</v>
+        <v>263</v>
       </c>
       <c r="E421" s="3" t="n">
         <v>21000</v>
@@ -12154,7 +12154,7 @@
         </is>
       </c>
       <c r="D422" s="2" t="n">
-        <v>-32</v>
+        <v>-38</v>
       </c>
       <c r="E422" s="3" t="n">
         <v>8000</v>
@@ -12182,7 +12182,7 @@
         </is>
       </c>
       <c r="D423" s="2" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E423" s="3" t="n">
         <v>21000</v>
@@ -12210,7 +12210,7 @@
         </is>
       </c>
       <c r="D424" s="2" t="n">
-        <v>-39</v>
+        <v>-57</v>
       </c>
       <c r="E424" s="3" t="n">
         <v>8000</v>
@@ -12238,7 +12238,7 @@
         </is>
       </c>
       <c r="D425" s="2" t="n">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="E425" s="3" t="n">
         <v>21000</v>
@@ -12378,7 +12378,7 @@
         </is>
       </c>
       <c r="D430" s="2" t="n">
-        <v>193</v>
+        <v>54</v>
       </c>
       <c r="E430" s="3" t="n">
         <v>6750</v>
@@ -12434,7 +12434,7 @@
         </is>
       </c>
       <c r="D432" s="2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E432" s="3" t="n">
         <v>2500</v>
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="D442" s="2" t="n">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="E442" s="3" t="n">
         <v>3500</v>
@@ -12770,7 +12770,7 @@
         </is>
       </c>
       <c r="D444" s="2" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="E444" s="3" t="n">
         <v>2500</v>
@@ -12826,7 +12826,7 @@
         </is>
       </c>
       <c r="D446" s="2" t="n">
-        <v>4563</v>
+        <v>4527</v>
       </c>
       <c r="E446" s="3" t="n">
         <v>2500</v>
@@ -13050,7 +13050,7 @@
         </is>
       </c>
       <c r="D454" s="2" t="n">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="E454" s="3" t="n">
         <v>5000</v>
@@ -13078,7 +13078,7 @@
         </is>
       </c>
       <c r="D455" s="2" t="n">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E455" s="3" t="n">
         <v>5000</v>
@@ -13106,7 +13106,7 @@
         </is>
       </c>
       <c r="D456" s="2" t="n">
-        <v>307</v>
+        <v>111</v>
       </c>
       <c r="E456" s="3" t="n">
         <v>5000</v>
@@ -13190,7 +13190,7 @@
         </is>
       </c>
       <c r="D459" s="2" t="n">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="E459" s="3" t="n">
         <v>12758</v>
@@ -13218,7 +13218,7 @@
         </is>
       </c>
       <c r="D460" s="2" t="n">
-        <v>6027</v>
+        <v>6003</v>
       </c>
       <c r="E460" s="3" t="n">
         <v>7312</v>
@@ -13274,7 +13274,7 @@
         </is>
       </c>
       <c r="D462" s="2" t="n">
-        <v>1480</v>
+        <v>1468</v>
       </c>
       <c r="E462" s="3" t="n">
         <v>7390</v>
@@ -13358,7 +13358,7 @@
         </is>
       </c>
       <c r="D465" s="2" t="n">
-        <v>495</v>
+        <v>471</v>
       </c>
       <c r="E465" s="3" t="n">
         <v>9164</v>
@@ -14590,7 +14590,7 @@
         </is>
       </c>
       <c r="D509" s="2" t="n">
-        <v>1503</v>
+        <v>1497</v>
       </c>
       <c r="E509" s="3" t="n">
         <v>7845</v>
@@ -14842,7 +14842,7 @@
         </is>
       </c>
       <c r="D518" s="2" t="n">
-        <v>630</v>
+        <v>582</v>
       </c>
       <c r="E518" s="3" t="n">
         <v>12346</v>
@@ -14926,7 +14926,7 @@
         </is>
       </c>
       <c r="D521" s="2" t="n">
-        <v>1648</v>
+        <v>1636</v>
       </c>
       <c r="E521" s="3" t="n">
         <v>10295</v>
@@ -15010,7 +15010,7 @@
         </is>
       </c>
       <c r="D524" s="2" t="n">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="E524" s="3" t="n">
         <v>7139</v>
@@ -15066,7 +15066,7 @@
         </is>
       </c>
       <c r="D526" s="2" t="n">
-        <v>933</v>
+        <v>909</v>
       </c>
       <c r="E526" s="3" t="n">
         <v>6417</v>
@@ -15094,7 +15094,7 @@
         </is>
       </c>
       <c r="D527" s="2" t="n">
-        <v>2003</v>
+        <v>1997</v>
       </c>
       <c r="E527" s="3" t="n">
         <v>7174</v>
@@ -15122,7 +15122,7 @@
         </is>
       </c>
       <c r="D528" s="2" t="n">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="E528" s="3" t="n">
         <v>10733</v>
@@ -15178,7 +15178,7 @@
         </is>
       </c>
       <c r="D530" s="2" t="n">
-        <v>769</v>
+        <v>745</v>
       </c>
       <c r="E530" s="3" t="n">
         <v>10604</v>
@@ -15346,7 +15346,7 @@
         </is>
       </c>
       <c r="D536" s="2" t="n">
-        <v>3078</v>
+        <v>3054</v>
       </c>
       <c r="E536" s="3" t="n">
         <v>14699</v>
@@ -15626,7 +15626,7 @@
         </is>
       </c>
       <c r="D546" s="2" t="n">
-        <v>775</v>
+        <v>763</v>
       </c>
       <c r="E546" s="3" t="n">
         <v>10365</v>
@@ -15850,7 +15850,7 @@
         </is>
       </c>
       <c r="D554" s="2" t="n">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="E554" s="3" t="n">
         <v>11078</v>
@@ -15878,7 +15878,7 @@
         </is>
       </c>
       <c r="D555" s="2" t="n">
-        <v>770</v>
+        <v>758</v>
       </c>
       <c r="E555" s="3" t="n">
         <v>11491</v>
@@ -16074,7 +16074,7 @@
         </is>
       </c>
       <c r="D562" s="2" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E562" s="3" t="n">
         <v>12900</v>
@@ -16242,7 +16242,7 @@
         </is>
       </c>
       <c r="D568" s="2" t="n">
-        <v>4181</v>
+        <v>4169</v>
       </c>
       <c r="E568" s="3" t="n">
         <v>11094</v>
@@ -18874,7 +18874,7 @@
         </is>
       </c>
       <c r="D662" s="2" t="n">
-        <v>389</v>
+        <v>369</v>
       </c>
       <c r="E662" s="3" t="n">
         <v>1</v>
@@ -19574,7 +19574,7 @@
         </is>
       </c>
       <c r="D687" s="2" t="n">
-        <v>1262</v>
+        <v>1250</v>
       </c>
       <c r="E687" s="3" t="n">
         <v>12816</v>
@@ -19602,7 +19602,7 @@
         </is>
       </c>
       <c r="D688" s="2" t="n">
-        <v>907</v>
+        <v>877</v>
       </c>
       <c r="E688" s="3" t="n">
         <v>22302</v>
@@ -20134,7 +20134,7 @@
         </is>
       </c>
       <c r="D707" s="2" t="n">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E707" s="3" t="n">
         <v>26896</v>
@@ -20218,7 +20218,7 @@
         </is>
       </c>
       <c r="D710" s="2" t="n">
-        <v>570</v>
+        <v>558</v>
       </c>
       <c r="E710" s="3" t="n">
         <v>13500</v>
@@ -20386,7 +20386,7 @@
         </is>
       </c>
       <c r="D716" s="2" t="n">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E716" s="3" t="n">
         <v>21000</v>
@@ -20414,7 +20414,7 @@
         </is>
       </c>
       <c r="D717" s="2" t="n">
-        <v>445</v>
+        <v>425</v>
       </c>
       <c r="E717" s="3" t="n">
         <v>1</v>
@@ -21674,7 +21674,7 @@
         </is>
       </c>
       <c r="D762" s="2" t="n">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E762" s="3" t="n">
         <v>5243</v>
@@ -25594,7 +25594,7 @@
         </is>
       </c>
       <c r="D902" s="2" t="n">
-        <v>641</v>
+        <v>625</v>
       </c>
       <c r="E902" s="3" t="n">
         <v>26000</v>
@@ -25930,7 +25930,7 @@
         </is>
       </c>
       <c r="D914" s="2" t="n">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E914" s="3" t="n">
         <v>20000</v>
@@ -25958,7 +25958,7 @@
         </is>
       </c>
       <c r="D915" s="2" t="n">
-        <v>752</v>
+        <v>740</v>
       </c>
       <c r="E915" s="3" t="n">
         <v>12500</v>
@@ -26182,7 +26182,7 @@
         </is>
       </c>
       <c r="D923" s="2" t="n">
-        <v>1913</v>
+        <v>1853</v>
       </c>
       <c r="E923" s="3" t="n">
         <v>3800</v>
@@ -26238,7 +26238,7 @@
         </is>
       </c>
       <c r="D925" s="2" t="n">
-        <v>1379</v>
+        <v>1359</v>
       </c>
       <c r="E925" s="3" t="n">
         <v>1195</v>
@@ -32819,7 +32819,7 @@
         </is>
       </c>
       <c r="D1160" s="2" t="n">
-        <v>480</v>
+        <v>468</v>
       </c>
       <c r="E1160" s="3" t="n">
         <v>6329</v>
@@ -32847,7 +32847,7 @@
         </is>
       </c>
       <c r="D1161" s="2" t="n">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="E1161" s="3" t="n">
         <v>6737</v>
@@ -32875,7 +32875,7 @@
         </is>
       </c>
       <c r="D1162" s="2" t="n">
-        <v>612</v>
+        <v>600</v>
       </c>
       <c r="E1162" s="3" t="n">
         <v>6350</v>
@@ -32959,7 +32959,7 @@
         </is>
       </c>
       <c r="D1165" s="2" t="n">
-        <v>451</v>
+        <v>439</v>
       </c>
       <c r="E1165" s="3" t="n">
         <v>3900</v>

</xml_diff>